<commit_message>
Literature review matrix: on-this-page overview, stopping rule, explanatory columns, quotes sheet
Bold key words in the Scholar list, add a search-within-citing screenshot, move the worked example next to the tidy-data advice, rename treatment columns to explanatory in the page and the downloads, move quotes to their own sheet in the template, replace the writing section with advice on when to stop searching, add a new card image, and revise the prose.
</commit_message>
<xml_diff>
--- a/assets/files/lit-review-matrix-example.xlsx
+++ b/assets/files/lit-review-matrix-example.xlsx
@@ -500,12 +500,12 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>treatment</t>
+          <t>explanatory</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>treatment_measure</t>
+          <t>explanatory_measure</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Deploying to gh-pages from @ etjernst/etjernst.github.io@59aa745702bd6d6cbff6c0dc0dc687bc3f65fbab 🚀
</commit_message>
<xml_diff>
--- a/assets/files/lit-review-matrix-example.xlsx
+++ b/assets/files/lit-review-matrix-example.xlsx
@@ -500,12 +500,12 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>treatment</t>
+          <t>explanatory</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>treatment_measure</t>
+          <t>explanatory_measure</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Example matrix: consistent identification, pollutant, and field labels; smaller card titles on the resources page
</commit_message>
<xml_diff>
--- a/assets/files/lit-review-matrix-example.xlsx
+++ b/assets/files/lit-review-matrix-example.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Panel (but they refer to IV on p. 14)</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>1) Distinguishing the causal effects of air pollution on mortality from unobserved correlated confounding factors can be difficult (p. 3) 2) Details of distances of downwind dispersion plumes of pollutants: UFPM (570-910m), NO and NO2 (550-570m), CO, PM2.5, and PM10 (100-200m) 3) Studies show that without filtration systems, most homes are highly penetrated by UFP. 4) Though there are limited controls used for differing populations, the study relies on comparing nearby, presumably similar, blocks which lie in different directions of wind-blown highway pollution. / Similar elements here to your proposed Nairobi experiment. Includes information about wind direction determination.</t>
+          <t>1) Distinguishing the causal effects of air pollution on mortality from unobserved correlated confounding factors can be difficult (p. 3) 2) Details of distances of downwind dispersion plumes of pollutants: UFPM (570-910m), NO and NO2 (550-570m), CO, PM2.5, and PM10 (100-200m) 3) Studies show that without filtration systems, most homes are highly penetrated by UFP. 4) Though there are limited controls used for differing populations, the study relies on comparing nearby, presumably similar, blocks which lie in different directions of wind-blown highway pollution. / Similar elements here to your proposed Nairobi experiment. Includes information about wind direction determination. / Identification: panel, though the authors refer to instrumental variables on p. 14.</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Instrumental Variable</t>
+          <t>Instrumental variables</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr"/>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
@@ -1251,12 +1251,12 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>Instrumental variables</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>TSP; TSPs</t>
+          <t>TSP</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Natural</t>
+          <t>Natural experiment</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>TSPs; dust</t>
+          <t>TSP; dust</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Instrumental Variable</t>
+          <t>Instrumental variables</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr"/>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Natural and Panel</t>
+          <t>Natural experiment; Panel</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>TSPs; NO2; CO</t>
+          <t>TSP; NO2; CO</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>PM10; O3; CO; Ozone</t>
+          <t>PM10; O3; CO</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>PM10; CO; ozone</t>
+          <t>PM10; CO; O3</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S15" s="2" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr"/>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Ordinary Least Squares AND Instrumental Variable</t>
+          <t>OLS; Instrumental variables</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S17" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S18" s="2" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>NO2; O3; ozone</t>
+          <t>NO2; O3</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S20" s="2" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S21" s="2" t="inlineStr"/>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr">
@@ -2523,12 +2523,12 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Natural?</t>
+          <t>Natural experiment?</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>ozone; aerosol</t>
+          <t>O3; aerosol</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Science, and Economic</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S23" s="2" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S24" s="2" t="inlineStr"/>
@@ -2711,12 +2711,12 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Panel (and also a qualitative survey)</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>PM2.5; Dust</t>
+          <t>PM2.5; dust</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2743,13 +2743,13 @@
       </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>1) This is an 82-page thesis. As such, there is much more information not included in this brief summary. 2) Document contains significant background information about air pollution, demographic trends, and more, in Kenya. 3) It is one of few studies measuring the perception of risks posed by air pollution in Kenya and wider Africa. 4) Air monitors used were found to overestimate PM2.5 levels and therefore a correction measure was necessary to correct (p. 22). / In depth paper. Provides much background on the topic of air pollution in Kenya. Also provides information about setting up cheap air sensors.</t>
+          <t>1) This is an 82-page thesis. As such, there is much more information not included in this brief summary. 2) Document contains significant background information about air pollution, demographic trends, and more, in Kenya. 3) It is one of few studies measuring the perception of risks posed by air pollution in Kenya and wider Africa. 4) Air monitors used were found to overestimate PM2.5 levels and therefore a correction measure was necessary to correct (p. 22). / In depth paper. Provides much background on the topic of air pollution in Kenya. Also provides information about setting up cheap air sensors. / Identification: panel, plus a qualitative survey.</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S26" s="2" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="R27" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S27" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>NO2; CO; Ozone</t>
+          <t>NO2; CO; O3</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S29" s="2" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S30" s="2" t="inlineStr"/>
@@ -3299,7 +3299,7 @@
       </c>
       <c r="R31" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S31" s="2" t="inlineStr">
@@ -3357,12 +3357,12 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Natural and Panel</t>
+          <t>Natural experiment; Panel</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>TSP; ozone; aerosol</t>
+          <t>TSP; O3; aerosol</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S32" s="2" t="inlineStr">
@@ -3451,12 +3451,12 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Studies reanalyzed were panel studies</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>PM 2.5; PM10; PM 2.1; PM; aerosols</t>
+          <t>PM2.5; PM10; PM2.1; PM; aerosol</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S33" s="2" t="inlineStr"/>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Natural</t>
+          <t>Natural experiment</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S34" s="2" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S35" s="2" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="R36" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S36" s="2" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S37" s="2" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>ozone</t>
+          <t>O3</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S38" s="2" t="inlineStr">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S39" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Deploying to gh-pages from @ etjernst/etjernst.github.io@5531cb5b41b9a6e10c128272cbf95ece7240e81e 🚀
</commit_message>
<xml_diff>
--- a/assets/files/lit-review-matrix-example.xlsx
+++ b/assets/files/lit-review-matrix-example.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Panel (but they refer to IV on p. 14)</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>1) Distinguishing the causal effects of air pollution on mortality from unobserved correlated confounding factors can be difficult (p. 3) 2) Details of distances of downwind dispersion plumes of pollutants: UFPM (570-910m), NO and NO2 (550-570m), CO, PM2.5, and PM10 (100-200m) 3) Studies show that without filtration systems, most homes are highly penetrated by UFP. 4) Though there are limited controls used for differing populations, the study relies on comparing nearby, presumably similar, blocks which lie in different directions of wind-blown highway pollution. / Similar elements here to your proposed Nairobi experiment. Includes information about wind direction determination.</t>
+          <t>1) Distinguishing the causal effects of air pollution on mortality from unobserved correlated confounding factors can be difficult (p. 3) 2) Details of distances of downwind dispersion plumes of pollutants: UFPM (570-910m), NO and NO2 (550-570m), CO, PM2.5, and PM10 (100-200m) 3) Studies show that without filtration systems, most homes are highly penetrated by UFP. 4) Though there are limited controls used for differing populations, the study relies on comparing nearby, presumably similar, blocks which lie in different directions of wind-blown highway pollution. / Similar elements here to your proposed Nairobi experiment. Includes information about wind direction determination. / Identification: panel, though the authors refer to instrumental variables on p. 14.</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Instrumental Variable</t>
+          <t>Instrumental variables</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr"/>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
@@ -1251,12 +1251,12 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>Instrumental variables</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>TSP; TSPs</t>
+          <t>TSP</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Natural</t>
+          <t>Natural experiment</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>TSPs; dust</t>
+          <t>TSP; dust</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Instrumental Variable</t>
+          <t>Instrumental variables</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr"/>
@@ -1619,12 +1619,12 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Natural and Panel</t>
+          <t>Natural experiment; Panel</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>TSPs; NO2; CO</t>
+          <t>TSP; NO2; CO</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>PM10; O3; CO; Ozone</t>
+          <t>PM10; O3; CO</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S14" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>PM10; CO; ozone</t>
+          <t>PM10; CO; O3</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S15" s="2" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S16" s="2" t="inlineStr"/>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Ordinary Least Squares AND Instrumental Variable</t>
+          <t>OLS; Instrumental variables</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S17" s="2" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S18" s="2" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S19" s="2" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>NO2; O3; ozone</t>
+          <t>NO2; O3</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S20" s="2" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S21" s="2" t="inlineStr"/>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S22" s="2" t="inlineStr">
@@ -2523,12 +2523,12 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Natural?</t>
+          <t>Natural experiment?</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>ozone; aerosol</t>
+          <t>O3; aerosol</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Science, and Economic</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S23" s="2" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S24" s="2" t="inlineStr"/>
@@ -2711,12 +2711,12 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Panel (and also a qualitative survey)</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>PM2.5; Dust</t>
+          <t>PM2.5; dust</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2743,13 +2743,13 @@
       </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>1) This is an 82-page thesis. As such, there is much more information not included in this brief summary. 2) Document contains significant background information about air pollution, demographic trends, and more, in Kenya. 3) It is one of few studies measuring the perception of risks posed by air pollution in Kenya and wider Africa. 4) Air monitors used were found to overestimate PM2.5 levels and therefore a correction measure was necessary to correct (p. 22). / In depth paper. Provides much background on the topic of air pollution in Kenya. Also provides information about setting up cheap air sensors.</t>
+          <t>1) This is an 82-page thesis. As such, there is much more information not included in this brief summary. 2) Document contains significant background information about air pollution, demographic trends, and more, in Kenya. 3) It is one of few studies measuring the perception of risks posed by air pollution in Kenya and wider Africa. 4) Air monitors used were found to overestimate PM2.5 levels and therefore a correction measure was necessary to correct (p. 22). / In depth paper. Provides much background on the topic of air pollution in Kenya. Also provides information about setting up cheap air sensors. / Identification: panel, plus a qualitative survey.</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S26" s="2" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="R27" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S27" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>NO2; CO; Ozone</t>
+          <t>NO2; CO; O3</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S28" s="2" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S29" s="2" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S30" s="2" t="inlineStr"/>
@@ -3299,7 +3299,7 @@
       </c>
       <c r="R31" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S31" s="2" t="inlineStr">
@@ -3357,12 +3357,12 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Natural and Panel</t>
+          <t>Natural experiment; Panel</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>TSP; ozone; aerosol</t>
+          <t>TSP; O3; aerosol</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S32" s="2" t="inlineStr">
@@ -3451,12 +3451,12 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Studies reanalyzed were panel studies</t>
+          <t>Panel</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>PM 2.5; PM10; PM 2.1; PM; aerosols</t>
+          <t>PM2.5; PM10; PM2.1; PM; aerosol</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S33" s="2" t="inlineStr"/>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Natural</t>
+          <t>Natural experiment</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S34" s="2" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>Public Health, Economics, and Science</t>
+          <t>Public health; economics; science</t>
         </is>
       </c>
       <c r="S35" s="2" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="R36" s="2" t="inlineStr">
         <is>
-          <t>Public health and science</t>
+          <t>Public health; science</t>
         </is>
       </c>
       <c r="S36" s="2" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S37" s="2" t="inlineStr">
@@ -3926,7 +3926,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>ozone</t>
+          <t>O3</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S38" s="2" t="inlineStr">
@@ -4019,7 +4019,7 @@
       </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>Public Health and Economics</t>
+          <t>Public health; economics</t>
         </is>
       </c>
       <c r="S39" s="2" t="inlineStr">

</xml_diff>